<commit_message>
sf10000 spread sheet with todays test results.
Former-commit-id: e5cb622954869eed85357852f69c22ac0f401131
</commit_message>
<xml_diff>
--- a/SF10000/LoadResultsSVR.xlsx
+++ b/SF10000/LoadResultsSVR.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="51200" windowHeight="26460" tabRatio="500"/>
+    <workbookView xWindow="1240" yWindow="1200" windowWidth="51200" windowHeight="26460" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
   <si>
     <t>PartitionsPerNode</t>
   </si>
@@ -180,6 +180,36 @@
   </si>
   <si>
     <t>311.8s</t>
+  </si>
+  <si>
+    <t>Entry optimizations(timing)</t>
+  </si>
+  <si>
+    <t>Entry optimizatuions (buffers_idx)</t>
+  </si>
+  <si>
+    <t>Entry optimizations  (buffers_hidden)</t>
+  </si>
+  <si>
+    <t>458.8s</t>
+  </si>
+  <si>
+    <t>Entry optimizations  (buffers idx) compact</t>
+  </si>
+  <si>
+    <t>time to compact</t>
+  </si>
+  <si>
+    <t>4262s</t>
+  </si>
+  <si>
+    <t>space</t>
+  </si>
+  <si>
+    <t>110gb</t>
+  </si>
+  <si>
+    <t>421s</t>
   </si>
 </sst>
 </file>
@@ -223,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -231,6 +261,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -510,9 +546,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:Z10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="6.1640625" customWidth="1"/>
     <col min="3" max="4" width="17.33203125" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
@@ -524,9 +561,14 @@
     <col min="14" max="15" width="21.33203125" style="2" customWidth="1"/>
     <col min="16" max="16" width="15.33203125" style="3" customWidth="1"/>
     <col min="17" max="17" width="16.5" style="3" customWidth="1"/>
+    <col min="21" max="21" width="11.83203125" style="2" customWidth="1"/>
+    <col min="22" max="22" width="14.5" customWidth="1"/>
+    <col min="23" max="23" width="14.6640625" customWidth="1"/>
+    <col min="24" max="24" width="13.5" style="4" customWidth="1"/>
+    <col min="25" max="26" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D1" t="s">
         <v>5</v>
       </c>
@@ -534,7 +576,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="96" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" ht="96" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -589,8 +631,26 @@
       <c r="S2" s="3" t="s">
         <v>47</v>
       </c>
+      <c r="U2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -637,7 +697,7 @@
         <v>30.3</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -684,7 +744,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>10</v>
       </c>
@@ -742,8 +802,20 @@
       <c r="T6" s="2" t="s">
         <v>50</v>
       </c>
+      <c r="U6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="V6">
+        <v>8881</v>
+      </c>
+      <c r="W6">
+        <v>4097</v>
+      </c>
+      <c r="X6" s="4">
+        <v>2409</v>
+      </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>10</v>
       </c>
@@ -794,6 +866,61 @@
       </c>
       <c r="T7" s="2" t="s">
         <v>49</v>
+      </c>
+      <c r="U7" s="2">
+        <v>44.6</v>
+      </c>
+      <c r="V7">
+        <v>8888</v>
+      </c>
+      <c r="W7">
+        <v>4112</v>
+      </c>
+      <c r="X7" s="4">
+        <v>2432</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z7" s="4">
+        <v>11.44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>100</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>100</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="V10">
+        <v>88135</v>
+      </c>
+      <c r="W10">
+        <v>32784</v>
+      </c>
+      <c r="X10" s="4">
+        <v>24110</v>
+      </c>
+      <c r="Y10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z10" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some more test results.
Former-commit-id: 79a26193ebec1812d434bf8f61ecc3809f7e1d43
</commit_message>
<xml_diff>
--- a/SF10000/LoadResultsSVR.xlsx
+++ b/SF10000/LoadResultsSVR.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="66">
   <si>
     <t>PartitionsPerNode</t>
   </si>
@@ -203,13 +203,28 @@
     <t>4262s</t>
   </si>
   <si>
-    <t>space</t>
-  </si>
-  <si>
-    <t>110gb</t>
-  </si>
-  <si>
     <t>421s</t>
+  </si>
+  <si>
+    <t>11.44gb</t>
+  </si>
+  <si>
+    <t>space itemSize i3</t>
+  </si>
+  <si>
+    <t>space itemSize i4</t>
+  </si>
+  <si>
+    <t>11.56gb</t>
+  </si>
+  <si>
+    <t>110.4gb</t>
+  </si>
+  <si>
+    <t>time to compact i4</t>
+  </si>
+  <si>
+    <t>358s</t>
   </si>
 </sst>
 </file>
@@ -546,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z10"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.1640625" customWidth="1"/>
@@ -565,10 +580,11 @@
     <col min="22" max="22" width="14.5" customWidth="1"/>
     <col min="23" max="23" width="14.6640625" customWidth="1"/>
     <col min="24" max="24" width="13.5" style="4" customWidth="1"/>
-    <col min="25" max="26" width="10.83203125" style="4"/>
+    <col min="25" max="27" width="10.83203125" style="4"/>
+    <col min="28" max="28" width="10.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
       <c r="D1" t="s">
         <v>5</v>
       </c>
@@ -576,7 +592,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="96" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:28" ht="96" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -647,10 +663,16 @@
         <v>56</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -697,7 +719,7 @@
         <v>30.3</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -744,7 +766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>10</v>
       </c>
@@ -814,8 +836,20 @@
       <c r="X6" s="4">
         <v>2409</v>
       </c>
+      <c r="Y6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z6" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB6" s="4" t="s">
+        <v>62</v>
+      </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>10</v>
       </c>
@@ -879,14 +913,8 @@
       <c r="X7" s="4">
         <v>2432</v>
       </c>
-      <c r="Y7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z7" s="4">
-        <v>11.44</v>
-      </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>100</v>
       </c>
@@ -897,7 +925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>100</v>
       </c>
@@ -920,7 +948,7 @@
         <v>57</v>
       </c>
       <c r="Z10" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>